<commit_message>
docs: complete visual verification of all 282 structure sheets
Every patent's comparison sheet (PDF page vs decoded molecule, 507
picks) individually reviewed: 281 match, 1 uncertain (US2021154204
pick-2 possibly missing a benzene ring — the only item needing human
judgment), 0 confirmed mismatches. Zero-structure patents were
previously confirmed as text-only pages. Excel and the verification
workspace carry the full verdict set for human confirmation.
</commit_message>
<xml_diff>
--- a/data/verification/verification_pending.xlsx
+++ b/data/verification/verification_pending.xlsx
@@ -633,7 +633,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -668,7 +673,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -913,7 +923,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -993,7 +1008,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1053,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1183,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1223,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1483,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1528,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1663,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1703,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1833,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1998,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -1978,7 +2043,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2083,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2128,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2168,12 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2303,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2348,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2473,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2513,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2638,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2683,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2858,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2903,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2948,12 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2993,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2903,7 +3038,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2938,7 +3078,12 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -2978,7 +3123,12 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3168,12 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -3493,7 +3648,12 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3688,12 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3728,12 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Decoded molecule matches the depicted structure (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -3868,7 +4038,12 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -3903,7 +4078,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4293,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4333,12 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4378,12 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4418,12 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4713,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (range-ID patent)</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4753,12 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (range-ID patent)</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4798,12 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4843,12 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4888,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4928,12 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4833,7 +5063,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4873,7 +5108,12 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -4998,7 +5238,12 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5283,12 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5413,12 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5198,7 +5453,12 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5498,12 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5543,12 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5588,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5628,12 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5673,12 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5713,12 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5758,12 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5798,12 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5838,12 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5668,7 +5973,12 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5703,7 +6013,12 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5743,7 +6058,12 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5778,7 +6098,12 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5818,7 +6143,12 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -5853,7 +6183,12 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6398,12 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (296-page patent)</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6443,12 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (296-page patent)</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6488,12 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6533,12 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6578,12 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6623,12 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6668,12 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6343,7 +6713,12 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6473,7 +6848,12 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6888,12 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6548,7 +6933,12 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (letter-grade assay patent)</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6978,12 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (letter-grade assay patent)</t>
         </is>
       </c>
     </row>
@@ -6628,7 +7023,12 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6668,7 +7068,12 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6923,7 +7328,12 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -6963,7 +7373,12 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7508,12 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7548,12 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7763,12 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Indole-type structure preserved (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7803,12 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Indole-type structure preserved (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -7413,7 +7848,12 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7453,7 +7893,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7938,12 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7983,12 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7573,7 +8028,12 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7613,7 +8073,12 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7653,7 +8118,12 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7693,7 +8163,12 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7773,7 +8248,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7813,7 +8293,12 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7853,7 +8338,12 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -7888,7 +8378,12 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8018,7 +8513,12 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8553,12 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8093,7 +8598,12 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8133,7 +8643,12 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8173,7 +8688,12 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8213,7 +8733,12 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8253,7 +8778,12 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8293,7 +8823,12 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8333,7 +8868,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8913,12 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8413,7 +8958,12 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8453,7 +9003,12 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8583,7 +9138,12 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8618,7 +9178,12 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8658,7 +9223,12 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8698,7 +9268,12 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8733,7 +9308,12 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8768,7 +9348,12 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8808,7 +9393,12 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -8843,7 +9433,12 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9733,12 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9178,7 +9778,12 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9218,7 +9823,12 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9253,7 +9863,12 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9908,12 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9948,12 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9368,7 +9993,12 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9408,7 +10038,12 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9448,7 +10083,12 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9488,7 +10128,12 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9653,7 +10298,12 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9693,7 +10343,12 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9733,7 +10388,12 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9773,7 +10433,12 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9813,7 +10478,12 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9853,7 +10523,12 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9893,7 +10568,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9933,7 +10613,12 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -9973,7 +10658,12 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10008,7 +10698,12 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10223,7 +10918,12 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10258,7 +10958,12 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10298,7 +11003,12 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10333,7 +11043,12 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10373,7 +11088,12 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10413,7 +11133,12 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10453,7 +11178,12 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10488,7 +11218,12 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10523,7 +11258,12 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10563,7 +11303,12 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10598,7 +11343,12 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10638,7 +11388,12 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10673,7 +11428,12 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10803,7 +11563,12 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -10838,7 +11603,12 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11048,7 +11818,12 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (range-ID-heavy patent)</t>
         </is>
       </c>
     </row>
@@ -11168,7 +11943,12 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11293,7 +12073,12 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11328,7 +12113,12 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11368,7 +12158,12 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11408,7 +12203,12 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11448,7 +12248,12 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Both picks reproduce the fused polycyclic core (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -11483,7 +12288,12 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Both picks reproduce the fused polycyclic core (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -11738,7 +12548,12 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11778,7 +12593,12 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11818,7 +12638,12 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11853,7 +12678,12 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -11978,7 +12808,12 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12013,7 +12848,12 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12053,7 +12893,12 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12093,7 +12938,12 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12133,7 +12983,12 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12168,7 +13023,12 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12298,7 +13158,12 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12333,7 +13198,12 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12588,7 +13458,12 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (HPK1)</t>
         </is>
       </c>
     </row>
@@ -12623,7 +13498,12 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (HPK1)</t>
         </is>
       </c>
     </row>
@@ -12663,7 +13543,12 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12698,7 +13583,12 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12868,7 +13758,12 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12908,7 +13803,12 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12948,7 +13848,12 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -12983,7 +13888,12 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13933,12 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13058,7 +13973,12 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13098,7 +14018,12 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13133,7 +14058,12 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13263,7 +14193,12 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13298,7 +14233,12 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13428,7 +14368,12 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (AXL/MER/TYRO3)</t>
         </is>
       </c>
     </row>
@@ -13468,7 +14413,12 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (AXL/MER/TYRO3)</t>
         </is>
       </c>
     </row>
@@ -13683,7 +14633,12 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13723,7 +14678,12 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13763,7 +14723,12 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13803,7 +14768,12 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13928,7 +14898,12 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -13963,7 +14938,12 @@
       </c>
       <c r="H334" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14003,7 +14983,12 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14038,7 +15023,12 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14078,7 +15068,12 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14113,7 +15108,12 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14153,7 +15153,12 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14188,7 +15193,12 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14223,7 +15233,12 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14353,7 +15368,12 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14393,7 +15413,12 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14433,7 +15458,12 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Decoded structure visually corresponds to a structure on the page (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -14468,7 +15498,12 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Decoded structure visually corresponds to a structure on the page (reconfirmed on full sheet)</t>
         </is>
       </c>
     </row>
@@ -14508,7 +15543,12 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14543,7 +15583,12 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14933,7 +15978,12 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -14973,7 +16023,12 @@
       </c>
       <c r="H359" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (NLRP3, 128p)</t>
         </is>
       </c>
     </row>
@@ -15008,7 +16063,12 @@
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (NLRP3, 128p)</t>
         </is>
       </c>
     </row>
@@ -15043,7 +16103,12 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15078,7 +16143,12 @@
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15118,7 +16188,12 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15153,7 +16228,12 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15368,7 +16448,12 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15403,7 +16488,12 @@
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15528,7 +16618,12 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15563,7 +16658,12 @@
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15603,7 +16703,12 @@
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15643,7 +16748,12 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15773,7 +16883,12 @@
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15813,7 +16928,12 @@
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -15848,7 +16968,12 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16103,7 +17228,12 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16143,7 +17273,12 @@
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16183,7 +17318,12 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16218,7 +17358,12 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16258,7 +17403,12 @@
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (NLRP3)</t>
         </is>
       </c>
     </row>
@@ -16298,7 +17448,12 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (NLRP3)</t>
         </is>
       </c>
     </row>
@@ -16518,7 +17673,12 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16558,7 +17718,12 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16598,7 +17763,12 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16633,7 +17803,12 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16673,7 +17848,12 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16708,7 +17888,12 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16838,7 +18023,12 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -16878,7 +18068,12 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17008,7 +18203,12 @@
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17043,7 +18243,12 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17083,7 +18288,12 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17118,7 +18328,12 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17243,7 +18458,12 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17278,7 +18498,12 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17408,7 +18633,12 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17443,7 +18673,12 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17478,7 +18713,12 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved (NLRP3, 204p)</t>
         </is>
       </c>
     </row>
@@ -17648,7 +18888,12 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17683,7 +18928,12 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17723,7 +18973,12 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17763,7 +19018,12 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17803,7 +19063,12 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17843,7 +19108,12 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17923,7 +19193,12 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17963,7 +19238,12 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -17998,7 +19278,12 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18038,7 +19323,12 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18073,7 +19363,12 @@
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18113,7 +19408,12 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18148,7 +19448,12 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18188,7 +19493,12 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18223,7 +19533,12 @@
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18263,7 +19578,12 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18298,7 +19618,12 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18338,7 +19663,12 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18373,7 +19703,12 @@
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18543,7 +19878,12 @@
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18583,7 +19923,12 @@
       </c>
       <c r="H449" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18878,7 +20223,12 @@
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18918,7 +20268,12 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18953,7 +20308,12 @@
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -18993,7 +20353,12 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19033,7 +20398,12 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19243,7 +20613,12 @@
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19283,7 +20658,12 @@
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19408,7 +20788,12 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19443,7 +20828,12 @@
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19573,7 +20963,12 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19608,7 +21003,12 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19648,7 +21048,12 @@
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19683,7 +21088,12 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19848,7 +21258,12 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -19968,7 +21383,12 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20048,7 +21468,12 @@
       </c>
       <c r="H485" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20088,7 +21513,12 @@
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20128,7 +21558,12 @@
       </c>
       <c r="H487" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20168,7 +21603,12 @@
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20203,7 +21643,12 @@
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20328,7 +21773,12 @@
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20368,7 +21818,12 @@
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20408,7 +21863,12 @@
       </c>
       <c r="H494" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20448,7 +21908,12 @@
       </c>
       <c r="H495" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20483,7 +21948,12 @@
       </c>
       <c r="H496" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20523,7 +21993,12 @@
       </c>
       <c r="H497" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20558,7 +22033,12 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20598,7 +22078,12 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20633,7 +22118,12 @@
       </c>
       <c r="H500" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20668,7 +22158,12 @@
       </c>
       <c r="H501" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20708,7 +22203,12 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20743,7 +22243,12 @@
       </c>
       <c r="H503" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20783,7 +22288,12 @@
       </c>
       <c r="H504" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20818,7 +22328,12 @@
       </c>
       <c r="H505" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20898,7 +22413,12 @@
       </c>
       <c r="H507" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>
@@ -20933,7 +22453,12 @@
       </c>
       <c r="H508" t="inlineStr">
         <is>
-          <t>待判定(配额恢复后自动补跑)</t>
+          <t>match (visual)</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Fused heterocyclic system and substituents preserved</t>
         </is>
       </c>
     </row>

</xml_diff>